<commit_message>
tokens number measured AtoA
</commit_message>
<xml_diff>
--- a/DependEval/results/task4/AtoA/python/claude-haiku-4-5-python/claude-haiku-4-5_predictions_scores.xlsx
+++ b/DependEval/results/task4/AtoA/python/claude-haiku-4-5-python/claude-haiku-4-5_predictions_scores.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[["got-your-back/fmbox.py", "got-your-back/labellang.py"], ["got-your-back/gyb.py"]]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results atoa claude haiku
</commit_message>
<xml_diff>
--- a/DependEval/results/task4/AtoA/python/claude-haiku-4-5-python/claude-haiku-4-5_predictions_scores.xlsx
+++ b/DependEval/results/task4/AtoA/python/claude-haiku-4-5-python/claude-haiku-4-5_predictions_scores.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[["got-your-back/fmbox.py", "got-your-back/gyb.py"], ["got-your-back/labellang.py", "got-your-back/gyb.py"]]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>